<commit_message>
Fix broken mail and website entries for 14 Gemeinden
</commit_message>
<xml_diff>
--- a/gemeinden_XLSX.xlsx
+++ b/gemeinden_XLSX.xlsx
@@ -1297,7 +1297,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>"post@kukmirn.bgld.gv.at</t>
+          <t>post@kukmirn.bgld.gv.at</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>post@woerterberg.bgld.gv.a</t>
+          <t>post@woerterberg.bgld.gv.at</t>
         </is>
       </c>
     </row>
@@ -3707,12 +3707,12 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>http://www.weingraben.at/</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>post@weingraben.bgld.gv.at</t>
         </is>
       </c>
     </row>
@@ -3822,12 +3822,12 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>https://www.grafenschachen.at/</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>post@grafenschachen.bgld.gv.at</t>
         </is>
       </c>
     </row>
@@ -4213,12 +4213,12 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>nope</t>
+          <t>https://www.gemeinde-rotenturm.at/</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>post@rotenturm-pinka.bgld.gv.at</t>
         </is>
       </c>
     </row>
@@ -4448,7 +4448,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>post@badersdorf.bgld.gv.at%0a</t>
+          <t>post@badersdorf.bgld.gv.at</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8542,7 @@
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>sekretariat@enzesfeld-lindabrunn.a</t>
+          <t>sekretariat@enzesfeld-lindabrunn.at</t>
         </is>
       </c>
     </row>
@@ -9871,12 +9871,12 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>https://andlersdorf.gem2go.at/</t>
         </is>
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>gemeinde-andlersdorf@aon.at</t>
         </is>
       </c>
     </row>
@@ -10170,12 +10170,12 @@
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>https://www.grosshofen.gv.at/</t>
         </is>
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>gemeinde@grosshofen.gv.at</t>
         </is>
       </c>
     </row>
@@ -21008,7 +21008,7 @@
       </c>
       <c r="E891" t="inlineStr">
         <is>
-          <t>E:gemeinde@haigermoos.ooe.gv.at</t>
+          <t>gemeinde@haigermoos.ooe.gv.at</t>
         </is>
       </c>
     </row>
@@ -25465,7 +25465,7 @@
       </c>
       <c r="D1085" t="inlineStr">
         <is>
-          <t>St. Thomas am Blasenstein</t>
+          <t>https://www.st-thomas.at/</t>
         </is>
       </c>
       <c r="E1085" t="inlineStr">
@@ -28092,7 +28092,7 @@
       </c>
       <c r="E1199" t="inlineStr">
         <is>
-          <t>gemeinde@gro√É¬É√Ç¬üraming.ooe.gv.at</t>
+          <t>gemeinde@grossraming.ooe.gv.at</t>
         </is>
       </c>
     </row>
@@ -31082,7 +31082,7 @@
       </c>
       <c r="E1329" t="inlineStr">
         <is>
-          <t>"info@bad-vigaun.at</t>
+          <t>info@bad-vigaun.at</t>
         </is>
       </c>
     </row>
@@ -37430,7 +37430,7 @@
       </c>
       <c r="E1605" t="inlineStr">
         <is>
-          <t>SanktKathreinamOffenegg</t>
+          <t>gde@st-kathrein-offenegg.gv.at</t>
         </is>
       </c>
     </row>

</xml_diff>